<commit_message>
Feature: Single Query Progress, Filter/Sort, and Fixes
</commit_message>
<xml_diff>
--- a/roster.xlsx
+++ b/roster.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\credit_scrawl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E571506-50A4-4BDB-AD2C-E9F2895F554A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF882D96-3061-43A7-AD91-64AC89AE1B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="2535" windowWidth="30900" windowHeight="16575" xr2:uid="{234DCDC2-D0ED-4C1C-A020-34E605B55573}"/>
+    <workbookView xWindow="6420" yWindow="7080" windowWidth="30900" windowHeight="16575" xr2:uid="{234DCDC2-D0ED-4C1C-A020-34E605B55573}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>員編</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -61,16 +61,82 @@
     <t>C004</t>
   </si>
   <si>
+    <t>C005</t>
+  </si>
+  <si>
+    <t>C007</t>
+  </si>
+  <si>
     <t>詹錦嬰</t>
   </si>
   <si>
+    <t>郭昭德</t>
+  </si>
+  <si>
+    <t>李金英</t>
+  </si>
+  <si>
     <t>P221335683</t>
   </si>
   <si>
+    <t>D220460893</t>
+  </si>
+  <si>
+    <t>E200977156</t>
+  </si>
+  <si>
     <t>057/08/09</t>
   </si>
   <si>
+    <t>056/12/13</t>
+  </si>
+  <si>
+    <t>043/02/10</t>
+  </si>
+  <si>
     <t>府城</t>
+  </si>
+  <si>
+    <t>鴻康</t>
+  </si>
+  <si>
+    <t>C010</t>
+  </si>
+  <si>
+    <t>C011</t>
+  </si>
+  <si>
+    <t>C014</t>
+  </si>
+  <si>
+    <t>吳燕芳</t>
+  </si>
+  <si>
+    <t>陳明玉</t>
+  </si>
+  <si>
+    <t>方聖雯</t>
+  </si>
+  <si>
+    <t>D220017141</t>
+  </si>
+  <si>
+    <t>D221176685</t>
+  </si>
+  <si>
+    <t>R222418325</t>
+  </si>
+  <si>
+    <t>052/04/19</t>
+  </si>
+  <si>
+    <t>054/04/30</t>
+  </si>
+  <si>
+    <t>055/09/22</t>
+  </si>
+  <si>
+    <t>謙益</t>
   </si>
 </sst>
 </file>
@@ -457,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0047DDA-4F3F-4FF0-A2DB-D5018EBE2910}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11.625" bestFit="1" customWidth="1"/>
@@ -486,16 +552,101 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>